<commit_message>
Added L' and t to the other raw datasets and made them preprocessed. Clairifd isfracture function in hysteresis_loops.py
</commit_message>
<xml_diff>
--- a/Data/raw/TST_Bernaert_2024-09_FA/TST_2024-09_FA_metadata.xlsx
+++ b/Data/raw/TST_Bernaert_2024-09_FA/TST_2024-09_FA_metadata.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\oros\Downloads\TST_Bernaert_2024-09_FA\TST_Bernaert_2024-09_FA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\oros\Desktop\dataset_upload\TST_Bernaert_2024-09_FA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEE2252F-7473-41AF-94D6-D8E05B99100A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2AA0788-3CFD-4A9B-9280-D9987C63216B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="15" windowWidth="20640" windowHeight="11040" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Experiment" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="100">
   <si>
     <t>General</t>
   </si>
@@ -327,6 +327,12 @@
   </si>
   <si>
     <t>Fiber Material</t>
+  </si>
+  <si>
+    <t>L'</t>
+  </si>
+  <si>
+    <t>t</t>
   </si>
 </sst>
 </file>
@@ -422,7 +428,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -471,11 +477,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -527,11 +544,34 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="8">
+  <dxfs count="10">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -673,23 +713,23 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>308162</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>261471</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>179294</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>1617934</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>65244</xdr:rowOff>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>464715</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>127939</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Picture 3">
+        <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FC0C11FC-D7EF-49B6-9CF8-E8BD18A71247}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C395155E-785B-4554-A7AA-5CBCD555A698}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -705,8 +745,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="23429633" y="3585883"/>
-          <a:ext cx="6096851" cy="3391373"/>
+          <a:off x="25616647" y="1957294"/>
+          <a:ext cx="5679186" cy="2167410"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1368,32 +1408,32 @@
     <mergeCell ref="Q1:AI1"/>
   </mergeCells>
   <conditionalFormatting sqref="E3">
-    <cfRule type="expression" dxfId="7" priority="6">
+    <cfRule type="expression" dxfId="9" priority="6">
       <formula>D3="QS"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F3 M3 AL3:AM3">
-    <cfRule type="expression" dxfId="6" priority="9">
+    <cfRule type="expression" dxfId="8" priority="9">
       <formula>$D$3="FA"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G3">
-    <cfRule type="expression" dxfId="5" priority="5">
+    <cfRule type="expression" dxfId="7" priority="5">
       <formula>D3="OT"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H3 N3">
-    <cfRule type="expression" dxfId="4" priority="3">
+    <cfRule type="expression" dxfId="6" priority="3">
       <formula>G3="Other"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I3">
-    <cfRule type="expression" dxfId="3" priority="7">
+    <cfRule type="expression" dxfId="5" priority="7">
       <formula>OR(E3="fracture", F3="fracture")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S3">
-    <cfRule type="expression" dxfId="2" priority="1">
+    <cfRule type="expression" dxfId="4" priority="1">
       <formula>Q3="Other polymers"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1454,7 +1494,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:M18"/>
+  <dimension ref="A1:O18"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22.33203125" style="3" customWidth="1"/>
@@ -1465,14 +1505,14 @@
     <col min="6" max="6" width="19.109375" style="3" customWidth="1"/>
     <col min="7" max="7" width="19.88671875" style="3" customWidth="1"/>
     <col min="8" max="8" width="20.5546875" style="3" customWidth="1"/>
-    <col min="9" max="9" width="20.109375" style="3" customWidth="1"/>
-    <col min="10" max="11" width="15.6640625" style="3" customWidth="1"/>
-    <col min="12" max="12" width="21.88671875" style="3" customWidth="1"/>
-    <col min="13" max="13" width="20" style="3" customWidth="1"/>
-    <col min="14" max="16384" width="8.6640625" style="3"/>
+    <col min="9" max="11" width="20.109375" style="3" customWidth="1"/>
+    <col min="12" max="13" width="15.6640625" style="3" customWidth="1"/>
+    <col min="14" max="14" width="21.88671875" style="3" customWidth="1"/>
+    <col min="15" max="15" width="20" style="3" customWidth="1"/>
+    <col min="16" max="16384" width="8.6640625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="15" t="s">
         <v>49</v>
       </c>
@@ -1482,22 +1522,24 @@
       </c>
       <c r="D1" s="18"/>
       <c r="E1" s="18"/>
-      <c r="F1" s="16" t="s">
+      <c r="F1" s="19" t="s">
         <v>50</v>
       </c>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="14" t="s">
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
+      <c r="K1" s="21"/>
+      <c r="L1" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="K1" s="14"/>
-      <c r="L1" s="17" t="s">
+      <c r="M1" s="14"/>
+      <c r="N1" s="17" t="s">
         <v>52</v>
       </c>
-      <c r="M1" s="17"/>
-    </row>
-    <row r="2" spans="1:13" ht="41.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="O1" s="17"/>
+    </row>
+    <row r="2" spans="1:15" ht="41.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>77</v>
       </c>
@@ -1526,19 +1568,25 @@
         <v>85</v>
       </c>
       <c r="J2" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="L2" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="K2" s="4" t="s">
+      <c r="M2" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="L2" s="4" t="s">
+      <c r="N2" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="M2" s="4" t="s">
+      <c r="O2" s="4" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -1564,88 +1612,90 @@
       <c r="I3" s="6">
         <v>68.59</v>
       </c>
-      <c r="J3" s="11"/>
-      <c r="K3" s="11"/>
-      <c r="L3" s="6">
+      <c r="J3" s="6"/>
+      <c r="K3" s="6"/>
+      <c r="L3" s="11"/>
+      <c r="M3" s="11"/>
+      <c r="N3" s="6">
         <v>35</v>
       </c>
-      <c r="M3" s="6">
+      <c r="O3" s="6">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
       <c r="B5" s="1"/>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
       <c r="B6" s="1"/>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>
       <c r="B7" s="1"/>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
       <c r="B8" s="1"/>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
       <c r="B9" s="1"/>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
       <c r="B10" s="1"/>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
       <c r="B11" s="1"/>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
       <c r="B12" s="1"/>
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
       <c r="B13" s="1"/>
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
       <c r="B14" s="1"/>
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
       <c r="B15" s="1"/>
       <c r="D15" s="1"/>
       <c r="E15" s="1"/>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
       <c r="B16" s="1"/>
       <c r="D16" s="1"/>
@@ -1666,11 +1716,11 @@
   </sheetData>
   <sheetProtection selectLockedCells="1" selectUnlockedCells="1"/>
   <mergeCells count="5">
-    <mergeCell ref="J1:K1"/>
     <mergeCell ref="L1:M1"/>
+    <mergeCell ref="N1:O1"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C1:E1"/>
-    <mergeCell ref="F1:I1"/>
+    <mergeCell ref="F1:K1"/>
   </mergeCells>
   <pageMargins left="0.70000000000000007" right="0.70000000000000007" top="0.75" bottom="0.75" header="0.51181102362204722" footer="0.51181102362204722"/>
   <pageSetup firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>

<commit_message>
Updated Joseph fatigue dataset with t and l_prime
</commit_message>
<xml_diff>
--- a/Data/raw/TST_Bernaert_2024-09_FA/TST_2024-09_FA_metadata.xlsx
+++ b/Data/raw/TST_Bernaert_2024-09_FA/TST_2024-09_FA_metadata.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\oros\Desktop\dataset_upload\TST_Bernaert_2024-09_FA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\oros\Desktop\epfl\site&amp;report\dataset_upload\TST_Bernaert_2024-09_FA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2AA0788-3CFD-4A9B-9280-D9987C63216B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2F87F3C-33E8-4A68-97D6-513FEE7D691A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="15" windowWidth="20640" windowHeight="11040" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -557,21 +557,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="10">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="8">
     <dxf>
       <fill>
         <patternFill>
@@ -1408,32 +1394,32 @@
     <mergeCell ref="Q1:AI1"/>
   </mergeCells>
   <conditionalFormatting sqref="E3">
-    <cfRule type="expression" dxfId="9" priority="6">
+    <cfRule type="expression" dxfId="7" priority="6">
       <formula>D3="QS"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F3 M3 AL3:AM3">
-    <cfRule type="expression" dxfId="8" priority="9">
+    <cfRule type="expression" dxfId="6" priority="9">
       <formula>$D$3="FA"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G3">
-    <cfRule type="expression" dxfId="7" priority="5">
+    <cfRule type="expression" dxfId="5" priority="5">
       <formula>D3="OT"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H3 N3">
-    <cfRule type="expression" dxfId="6" priority="3">
+    <cfRule type="expression" dxfId="4" priority="3">
       <formula>G3="Other"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I3">
-    <cfRule type="expression" dxfId="5" priority="7">
+    <cfRule type="expression" dxfId="3" priority="7">
       <formula>OR(E3="fracture", F3="fracture")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S3">
-    <cfRule type="expression" dxfId="4" priority="1">
+    <cfRule type="expression" dxfId="2" priority="1">
       <formula>Q3="Other polymers"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1613,7 +1599,9 @@
         <v>68.59</v>
       </c>
       <c r="J3" s="6"/>
-      <c r="K3" s="6"/>
+      <c r="K3" s="6">
+        <v>27.45</v>
+      </c>
       <c r="L3" s="11"/>
       <c r="M3" s="11"/>
       <c r="N3" s="6">

</xml_diff>